<commit_message>
Update packing list generation outputs and templates.
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/output/1.xlsx
+++ b/output/1.xlsx
@@ -648,26 +648,23 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1048,320 +1045,339 @@
   <dimension ref="C2:I31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col width="0.727272727272727" customWidth="1" style="6" min="1" max="1"/>
-    <col width="1.35454545454545" customWidth="1" style="6" min="2" max="2"/>
-    <col width="18" customWidth="1" style="6" min="5" max="5"/>
-    <col width="22.7272727272727" customWidth="1" style="6" min="9" max="9"/>
+    <col hidden="1" width="0.727272727272727" customWidth="1" style="1" min="1" max="1"/>
+    <col width="0.454545454545455" customWidth="1" style="1" min="2" max="2"/>
+    <col width="5.36363636363636" customWidth="1" style="1" min="3" max="3"/>
+    <col width="38.3636363636364" customWidth="1" style="1" min="5" max="5"/>
+    <col width="5.72727272727273" customWidth="1" style="1" min="6" max="6"/>
+    <col width="7.18181818181818" customWidth="1" style="1" min="7" max="7"/>
+    <col width="8.36363636363636" customWidth="1" style="1" min="8" max="8"/>
+    <col width="9.72727272727273" customWidth="1" style="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="103" customHeight="1" s="6"/>
-    <row r="2" ht="30" customHeight="1" s="6">
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                              嘉兴凯实生物科技股份有限公司装箱单</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1" s="6">
+    <row r="1" ht="66" customHeight="1" s="1"/>
+    <row r="2" ht="30" customHeight="1" s="1">
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            嘉兴凯实生物科技股份有限公司装箱单</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1" s="1">
       <c r="C3" s="0" t="inlineStr">
         <is>
           <t>PO:</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1" s="6">
-      <c r="C4" s="2" t="inlineStr">
+    <row r="4" ht="24" customHeight="1" s="1">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>NO.</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve"> 料号/Part Number</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>名称/Description</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>批次</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>批次/Batch</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>版本/Edition</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>数量/Quantity</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>备注/Descr</t>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>备注/Remarks</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>17000050</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>垃圾桶</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="n"/>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>17000060</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>STRU-Cart垃圾桶-ODBC：DRW-Part-ODBC-0006</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="n"/>
     </row>
     <row r="6">
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="5" t="n"/>
+      <c r="C6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>17000060</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>STRU-Cart垃圾桶-ODBC：DRW-Part-ODBC-0006</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>5C01</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
+      <c r="C7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>17000610</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>STRU-阻燃棉-ODBC：DRW-Part-ODBC-0061</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>6401</v>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="I7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="C8" s="3" t="n"/>
+      <c r="C8" s="4" t="n"/>
       <c r="D8" s="5" t="n"/>
       <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
+      <c r="F8" s="0" t="n"/>
+      <c r="G8" s="0" t="n"/>
       <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
+      <c r="I8" s="0" t="n"/>
     </row>
     <row r="9">
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
+      <c r="C9" s="4" t="n"/>
+      <c r="E9" s="0" t="n"/>
+      <c r="F9" s="0" t="n"/>
+      <c r="G9" s="0" t="n"/>
+      <c r="H9" s="0" t="n"/>
+      <c r="I9" s="0" t="n"/>
     </row>
     <row r="10">
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
+      <c r="C10" s="4" t="n"/>
+      <c r="E10" s="0" t="n"/>
+      <c r="F10" s="0" t="n"/>
+      <c r="G10" s="0" t="n"/>
+      <c r="H10" s="0" t="n"/>
+      <c r="I10" s="0" t="n"/>
     </row>
     <row r="11">
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
+      <c r="C11" s="4" t="n"/>
+      <c r="E11" s="0" t="n"/>
+      <c r="F11" s="0" t="n"/>
+      <c r="G11" s="0" t="n"/>
+      <c r="H11" s="0" t="n"/>
+      <c r="I11" s="0" t="n"/>
     </row>
     <row r="12">
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
+      <c r="C12" s="4" t="n"/>
+      <c r="E12" s="0" t="n"/>
+      <c r="F12" s="0" t="n"/>
+      <c r="G12" s="0" t="n"/>
+      <c r="H12" s="0" t="n"/>
+      <c r="I12" s="0" t="n"/>
     </row>
     <row r="13">
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
+      <c r="C13" s="4" t="n"/>
+      <c r="E13" s="0" t="n"/>
+      <c r="F13" s="0" t="n"/>
+      <c r="G13" s="0" t="n"/>
+      <c r="H13" s="0" t="n"/>
+      <c r="I13" s="0" t="n"/>
     </row>
     <row r="14">
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="5" t="n"/>
+      <c r="C14" s="4" t="n"/>
+      <c r="E14" s="0" t="n"/>
+      <c r="F14" s="0" t="n"/>
+      <c r="G14" s="0" t="n"/>
+      <c r="H14" s="0" t="n"/>
+      <c r="I14" s="0" t="n"/>
     </row>
     <row r="15">
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
-      <c r="I15" s="5" t="n"/>
+      <c r="C15" s="4" t="n"/>
+      <c r="E15" s="0" t="n"/>
+      <c r="F15" s="0" t="n"/>
+      <c r="G15" s="0" t="n"/>
+      <c r="H15" s="0" t="n"/>
+      <c r="I15" s="0" t="n"/>
     </row>
     <row r="16">
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="5" t="n"/>
+      <c r="C16" s="4" t="n"/>
+      <c r="E16" s="0" t="n"/>
+      <c r="F16" s="0" t="n"/>
+      <c r="G16" s="0" t="n"/>
+      <c r="H16" s="0" t="n"/>
+      <c r="I16" s="0" t="n"/>
     </row>
     <row r="17">
-      <c r="C17" s="3" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="n"/>
+      <c r="C17" s="4" t="n"/>
+      <c r="E17" s="0" t="n"/>
+      <c r="F17" s="0" t="n"/>
+      <c r="G17" s="0" t="n"/>
+      <c r="H17" s="0" t="n"/>
+      <c r="I17" s="0" t="n"/>
     </row>
     <row r="18">
-      <c r="C18" s="3" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="n"/>
-      <c r="I18" s="5" t="n"/>
+      <c r="C18" s="4" t="n"/>
+      <c r="E18" s="0" t="n"/>
+      <c r="F18" s="0" t="n"/>
+      <c r="G18" s="0" t="n"/>
+      <c r="H18" s="0" t="n"/>
+      <c r="I18" s="0" t="n"/>
     </row>
     <row r="19">
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="5" t="n"/>
-      <c r="I19" s="5" t="n"/>
+      <c r="C19" s="4" t="n"/>
+      <c r="E19" s="0" t="n"/>
+      <c r="F19" s="0" t="n"/>
+      <c r="G19" s="0" t="n"/>
+      <c r="H19" s="0" t="n"/>
+      <c r="I19" s="0" t="n"/>
     </row>
     <row r="20">
-      <c r="C20" s="3" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="n"/>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="5" t="n"/>
-      <c r="I20" s="5" t="n"/>
+      <c r="C20" s="4" t="n"/>
+      <c r="E20" s="0" t="n"/>
+      <c r="F20" s="0" t="n"/>
+      <c r="G20" s="0" t="n"/>
+      <c r="H20" s="0" t="n"/>
+      <c r="I20" s="0" t="n"/>
     </row>
     <row r="21">
-      <c r="C21" s="3" t="n"/>
-      <c r="D21" s="5" t="n"/>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21" s="5" t="n"/>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="5" t="n"/>
-      <c r="I21" s="5" t="n"/>
+      <c r="C21" s="4" t="n"/>
+      <c r="E21" s="0" t="n"/>
+      <c r="F21" s="0" t="n"/>
+      <c r="G21" s="0" t="n"/>
+      <c r="H21" s="0" t="n"/>
+      <c r="I21" s="0" t="n"/>
     </row>
     <row r="22">
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="5" t="n"/>
-      <c r="E22" s="5" t="n"/>
-      <c r="F22" s="5" t="n"/>
-      <c r="G22" s="5" t="n"/>
-      <c r="H22" s="5" t="n"/>
-      <c r="I22" s="5" t="n"/>
+      <c r="C22" s="4" t="n"/>
+      <c r="E22" s="0" t="n"/>
+      <c r="F22" s="0" t="n"/>
+      <c r="G22" s="0" t="n"/>
+      <c r="H22" s="0" t="n"/>
+      <c r="I22" s="0" t="n"/>
     </row>
     <row r="23">
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="5" t="n"/>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="5" t="n"/>
-      <c r="I23" s="5" t="n"/>
+      <c r="C23" s="4" t="n"/>
+      <c r="E23" s="0" t="n"/>
+      <c r="F23" s="0" t="n"/>
+      <c r="G23" s="0" t="n"/>
+      <c r="H23" s="0" t="n"/>
+      <c r="I23" s="0" t="n"/>
     </row>
     <row r="24">
-      <c r="C24" s="3" t="n"/>
-      <c r="D24" s="5" t="n"/>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="5" t="n"/>
-      <c r="G24" s="5" t="n"/>
-      <c r="H24" s="5" t="n"/>
-      <c r="I24" s="5" t="n"/>
+      <c r="C24" s="4" t="n"/>
+      <c r="E24" s="0" t="n"/>
+      <c r="F24" s="0" t="n"/>
+      <c r="G24" s="0" t="n"/>
+      <c r="H24" s="0" t="n"/>
+      <c r="I24" s="0" t="n"/>
     </row>
     <row r="25">
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="5" t="n"/>
-      <c r="E25" s="5" t="n"/>
-      <c r="F25" s="5" t="n"/>
-      <c r="G25" s="5" t="n"/>
-      <c r="H25" s="5" t="n"/>
-      <c r="I25" s="5" t="n"/>
+      <c r="C25" s="4" t="n"/>
+      <c r="E25" s="0" t="n"/>
+      <c r="F25" s="0" t="n"/>
+      <c r="G25" s="0" t="n"/>
+      <c r="H25" s="0" t="n"/>
+      <c r="I25" s="0" t="n"/>
     </row>
     <row r="26">
-      <c r="C26" s="3" t="n"/>
-      <c r="D26" s="5" t="n"/>
-      <c r="E26" s="5" t="n"/>
-      <c r="F26" s="5" t="n"/>
-      <c r="G26" s="5" t="n"/>
-      <c r="H26" s="5" t="n"/>
-      <c r="I26" s="5" t="n"/>
+      <c r="C26" s="4" t="n"/>
+      <c r="E26" s="0" t="n"/>
+      <c r="F26" s="0" t="n"/>
+      <c r="G26" s="0" t="n"/>
+      <c r="H26" s="0" t="n"/>
+      <c r="I26" s="0" t="n"/>
     </row>
     <row r="27">
-      <c r="C27" s="3" t="n"/>
-      <c r="D27" s="5" t="n"/>
-      <c r="E27" s="5" t="n"/>
-      <c r="F27" s="5" t="n"/>
-      <c r="G27" s="5" t="n"/>
-      <c r="H27" s="5" t="n"/>
-      <c r="I27" s="5" t="n"/>
+      <c r="C27" s="4" t="n"/>
+      <c r="E27" s="0" t="n"/>
+      <c r="F27" s="0" t="n"/>
+      <c r="G27" s="0" t="n"/>
+      <c r="H27" s="0" t="n"/>
+      <c r="I27" s="0" t="n"/>
     </row>
     <row r="28">
-      <c r="C28" s="3" t="n"/>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="n"/>
-      <c r="G28" s="5" t="n"/>
-      <c r="H28" s="5" t="n"/>
-      <c r="I28" s="5" t="n"/>
+      <c r="C28" s="4" t="n"/>
+      <c r="E28" s="0" t="n"/>
+      <c r="F28" s="0" t="n"/>
+      <c r="G28" s="0" t="n"/>
+      <c r="H28" s="0" t="n"/>
+      <c r="I28" s="0" t="n"/>
     </row>
     <row r="29">
-      <c r="C29" s="3" t="n"/>
-      <c r="D29" s="5" t="n"/>
-      <c r="E29" s="5" t="n"/>
-      <c r="F29" s="5" t="n"/>
-      <c r="G29" s="5" t="n"/>
-      <c r="H29" s="5" t="n"/>
-      <c r="I29" s="5" t="n"/>
+      <c r="C29" s="4" t="n"/>
+      <c r="E29" s="0" t="n"/>
+      <c r="F29" s="0" t="n"/>
+      <c r="G29" s="0" t="n"/>
+      <c r="H29" s="0" t="n"/>
+      <c r="I29" s="0" t="n"/>
     </row>
     <row r="30">
-      <c r="C30" s="3" t="n"/>
-      <c r="D30" s="5" t="n"/>
-      <c r="E30" s="5" t="n"/>
-      <c r="F30" s="5" t="n"/>
-      <c r="G30" s="5" t="n"/>
-      <c r="H30" s="5" t="n"/>
-      <c r="I30" s="5" t="n"/>
+      <c r="C30" s="4" t="n"/>
+      <c r="E30" s="0" t="n"/>
+      <c r="F30" s="0" t="n"/>
+      <c r="G30" s="0" t="n"/>
+      <c r="H30" s="0" t="n"/>
+      <c r="I30" s="0" t="n"/>
     </row>
     <row r="31">
-      <c r="C31" s="3" t="n"/>
-      <c r="D31" s="5" t="n"/>
-      <c r="E31" s="5" t="n"/>
-      <c r="F31" s="5" t="n"/>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="5" t="n"/>
-      <c r="I31" s="5" t="n"/>
+      <c r="C31" s="4" t="n"/>
+      <c r="E31" s="0" t="n"/>
+      <c r="F31" s="0" t="n"/>
+      <c r="G31" s="0" t="n"/>
+      <c r="H31" s="0" t="n"/>
+      <c r="I31" s="0" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update app logic and refresh generated packing files.
Adjust app behavior and synchronize Excel templates/output artifacts with the latest packing list generation results.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/output/1.xlsx
+++ b/output/1.xlsx
@@ -1048,7 +1048,7 @@
     <col hidden="1" width="0.727272727272727" customWidth="1" style="1" min="1" max="1"/>
     <col width="0.454545454545455" customWidth="1" style="1" min="2" max="2"/>
     <col width="5.36363636363636" customWidth="1" style="1" min="3" max="3"/>
-    <col width="38.3636363636364" customWidth="1" style="1" min="5" max="5"/>
+    <col width="52.8181818181818" customWidth="1" style="1" min="5" max="5"/>
     <col width="5.72727272727273" customWidth="1" style="1" min="6" max="6"/>
     <col width="7.18181818181818" customWidth="1" style="1" min="7" max="7"/>
     <col width="8.36363636363636" customWidth="1" style="1" min="8" max="8"/>
@@ -1101,11 +1101,6 @@
           <t>数量/Quantity</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>备注/Remarks</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="C5" s="4" t="n">
@@ -1113,118 +1108,92 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>17000060</t>
+          <t>17008850</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>STRU-Cart垃圾桶-ODBC：DRW-Part-ODBC-0006</t>
+          <t>SLSU-湿度保温棉2-ODBC：DRW-Part-ODBC-0885</t>
         </is>
       </c>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>6301</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>V3</t>
+        </is>
+      </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I5" s="4" t="n"/>
     </row>
     <row r="6">
-      <c r="C6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>17000060</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>STRU-Cart垃圾桶-ODBC：DRW-Part-ODBC-0006</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>5C01</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>V2</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="5" t="n"/>
     </row>
     <row r="7">
-      <c r="C7" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>17000610</v>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>STRU-阻燃棉-ODBC：DRW-Part-ODBC-0061</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>6401</v>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>V1</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="I7" s="5" t="inlineStr"/>
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n"/>
+      <c r="I7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="C8" s="4" t="n"/>
       <c r="D8" s="5" t="n"/>
       <c r="E8" s="5" t="n"/>
-      <c r="F8" s="0" t="n"/>
-      <c r="G8" s="0" t="n"/>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="n"/>
       <c r="I8" s="0" t="n"/>
     </row>
     <row r="9">
       <c r="C9" s="4" t="n"/>
-      <c r="E9" s="0" t="n"/>
-      <c r="F9" s="0" t="n"/>
-      <c r="G9" s="0" t="n"/>
-      <c r="H9" s="0" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
       <c r="I9" s="0" t="n"/>
     </row>
     <row r="10">
       <c r="C10" s="4" t="n"/>
-      <c r="E10" s="0" t="n"/>
-      <c r="F10" s="0" t="n"/>
-      <c r="G10" s="0" t="n"/>
-      <c r="H10" s="0" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n"/>
       <c r="I10" s="0" t="n"/>
     </row>
     <row r="11">
       <c r="C11" s="4" t="n"/>
-      <c r="E11" s="0" t="n"/>
-      <c r="F11" s="0" t="n"/>
-      <c r="G11" s="0" t="n"/>
-      <c r="H11" s="0" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="n"/>
       <c r="I11" s="0" t="n"/>
     </row>
     <row r="12">
       <c r="C12" s="4" t="n"/>
-      <c r="E12" s="0" t="n"/>
-      <c r="F12" s="0" t="n"/>
-      <c r="G12" s="0" t="n"/>
-      <c r="H12" s="0" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="5" t="n"/>
       <c r="I12" s="0" t="n"/>
     </row>
     <row r="13">

</xml_diff>